<commit_message>
added new league and set for local
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -6,7 +6,7 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Overall STANDARD" r:id="rId3" sheetId="1"/>
+    <sheet name="Overall OBP" r:id="rId3" sheetId="1"/>
   </sheets>
 </workbook>
 </file>
@@ -32,40 +32,40 @@
     <t/>
   </si>
   <si>
-    <t>Jags In 2023</t>
-  </si>
-  <si>
-    <t>Feeling Ucey</t>
-  </si>
-  <si>
-    <t>Walks and Balks</t>
-  </si>
-  <si>
-    <t>IALO</t>
-  </si>
-  <si>
-    <t>Ever Dream</t>
-  </si>
-  <si>
-    <t>Slobber Knockers</t>
-  </si>
-  <si>
-    <t>Steel Wheels</t>
-  </si>
-  <si>
-    <t>Kansas City BBQ</t>
-  </si>
-  <si>
-    <t>The Black Hole</t>
-  </si>
-  <si>
-    <t>Apple Pie</t>
-  </si>
-  <si>
-    <t>𝙍 𝙊 𝘾 𝙆 ®</t>
-  </si>
-  <si>
-    <t>Reno Giants 2</t>
+    <t>What Did Yusei</t>
+  </si>
+  <si>
+    <t>Moonshots Only Club</t>
+  </si>
+  <si>
+    <t>Mitch</t>
+  </si>
+  <si>
+    <t>Mud Baez</t>
+  </si>
+  <si>
+    <t>The Vladiators</t>
+  </si>
+  <si>
+    <t>Maker of Rain</t>
+  </si>
+  <si>
+    <t>Salt Lake Bees</t>
+  </si>
+  <si>
+    <t>The Sandlot ⚾️</t>
+  </si>
+  <si>
+    <t>There's always next year</t>
+  </si>
+  <si>
+    <t>East Bound and Down</t>
+  </si>
+  <si>
+    <t>The Wolfpack</t>
+  </si>
+  <si>
+    <t>La Piedra</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -156,13 +156,13 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>82.5</v>
+        <v>111.0</v>
       </c>
       <c r="D2" t="n">
-        <v>47.5</v>
+        <v>46.0</v>
       </c>
       <c r="E2" t="n">
-        <v>35.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="3">
@@ -173,13 +173,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>79.0</v>
+        <v>107.0</v>
       </c>
       <c r="D3" t="n">
-        <v>32.5</v>
+        <v>54.5</v>
       </c>
       <c r="E3" t="n">
-        <v>46.5</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="4">
@@ -190,13 +190,13 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>77.5</v>
+        <v>98.0</v>
       </c>
       <c r="D4" t="n">
-        <v>38.0</v>
+        <v>62.0</v>
       </c>
       <c r="E4" t="n">
-        <v>39.5</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="5">
@@ -207,13 +207,13 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>75.0</v>
+        <v>89.5</v>
       </c>
       <c r="D5" t="n">
-        <v>43.0</v>
+        <v>50.0</v>
       </c>
       <c r="E5" t="n">
-        <v>32.0</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="6">
@@ -224,47 +224,47 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>70.5</v>
+        <v>86.0</v>
       </c>
       <c r="D6" t="n">
-        <v>26.0</v>
+        <v>34.5</v>
       </c>
       <c r="E6" t="n">
-        <v>44.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6.5</v>
+        <v>6.0</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>63.0</v>
+        <v>79.5</v>
       </c>
       <c r="D7" t="n">
-        <v>43.0</v>
+        <v>37.5</v>
       </c>
       <c r="E7" t="n">
-        <v>20.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6.5</v>
+        <v>7.0</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>63.0</v>
+        <v>76.0</v>
       </c>
       <c r="D8" t="n">
-        <v>41.0</v>
+        <v>40.0</v>
       </c>
       <c r="E8" t="n">
-        <v>22.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="9">
@@ -275,13 +275,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>61.5</v>
+        <v>73.5</v>
       </c>
       <c r="D9" t="n">
-        <v>37.0</v>
+        <v>35.5</v>
       </c>
       <c r="E9" t="n">
-        <v>24.5</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="10">
@@ -292,13 +292,13 @@
         <v>14</v>
       </c>
       <c r="C10" t="n">
-        <v>59.0</v>
+        <v>72.0</v>
       </c>
       <c r="D10" t="n">
-        <v>20.5</v>
+        <v>25.0</v>
       </c>
       <c r="E10" t="n">
-        <v>38.5</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="11">
@@ -312,10 +312,10 @@
         <v>53.0</v>
       </c>
       <c r="D11" t="n">
-        <v>29.5</v>
+        <v>28.0</v>
       </c>
       <c r="E11" t="n">
-        <v>23.5</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="12">
@@ -326,13 +326,13 @@
         <v>16</v>
       </c>
       <c r="C12" t="n">
-        <v>51.5</v>
+        <v>45.5</v>
       </c>
       <c r="D12" t="n">
-        <v>11.0</v>
+        <v>30.0</v>
       </c>
       <c r="E12" t="n">
-        <v>40.5</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="13">
@@ -343,13 +343,13 @@
         <v>17</v>
       </c>
       <c r="C13" t="n">
-        <v>44.5</v>
+        <v>45.0</v>
       </c>
       <c r="D13" t="n">
-        <v>21.0</v>
+        <v>25.0</v>
       </c>
       <c r="E13" t="n">
-        <v>23.5</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="14"/>
@@ -381,62 +381,62 @@
         <v>1.0</v>
       </c>
       <c r="B16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>47.5</v>
+        <v>62.0</v>
       </c>
       <c r="D16"/>
       <c r="E16" t="n">
         <v>1.0</v>
       </c>
       <c r="F16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G16" t="n">
-        <v>46.5</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2.5</v>
+        <v>2.0</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
-        <v>43.0</v>
+        <v>54.5</v>
       </c>
       <c r="D17"/>
       <c r="E17" t="n">
         <v>2.0</v>
       </c>
       <c r="F17" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G17" t="n">
-        <v>44.5</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C18" t="n">
-        <v>43.0</v>
+        <v>50.0</v>
       </c>
       <c r="D18"/>
       <c r="E18" t="n">
         <v>3.0</v>
       </c>
       <c r="F18" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>40.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="19">
@@ -444,20 +444,20 @@
         <v>4.0</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>41.0</v>
+        <v>46.0</v>
       </c>
       <c r="D19"/>
       <c r="E19" t="n">
         <v>4.0</v>
       </c>
       <c r="F19" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G19" t="n">
-        <v>39.5</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="20">
@@ -465,20 +465,20 @@
         <v>5.0</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
-        <v>38.0</v>
+        <v>40.0</v>
       </c>
       <c r="D20"/>
       <c r="E20" t="n">
         <v>5.0</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G20" t="n">
-        <v>38.5</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="21">
@@ -486,20 +486,20 @@
         <v>6.0</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n">
-        <v>37.0</v>
+        <v>37.5</v>
       </c>
       <c r="D21"/>
       <c r="E21" t="n">
         <v>6.0</v>
       </c>
       <c r="F21" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G21" t="n">
-        <v>35.0</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="22">
@@ -507,20 +507,20 @@
         <v>7.0</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C22" t="n">
-        <v>32.5</v>
+        <v>35.5</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="n">
         <v>7.0</v>
       </c>
       <c r="F22" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G22" t="n">
-        <v>32.0</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="23">
@@ -528,20 +528,20 @@
         <v>8.0</v>
       </c>
       <c r="B23" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>29.5</v>
+        <v>34.5</v>
       </c>
       <c r="D23"/>
       <c r="E23" t="n">
-        <v>8.0</v>
+        <v>8.5</v>
       </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G23" t="n">
-        <v>24.5</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="24">
@@ -549,20 +549,20 @@
         <v>9.0</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C24" t="n">
-        <v>26.0</v>
+        <v>30.0</v>
       </c>
       <c r="D24"/>
       <c r="E24" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="F24" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G24" t="n">
-        <v>23.5</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="25">
@@ -570,62 +570,62 @@
         <v>10.0</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C25" t="n">
-        <v>21.0</v>
+        <v>28.0</v>
       </c>
       <c r="D25"/>
       <c r="E25" t="n">
-        <v>9.5</v>
+        <v>10.0</v>
       </c>
       <c r="F25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G25" t="n">
-        <v>23.5</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>11.0</v>
+        <v>11.5</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
       </c>
       <c r="C26" t="n">
-        <v>20.5</v>
+        <v>25.0</v>
       </c>
       <c r="D26"/>
       <c r="E26" t="n">
         <v>11.0</v>
       </c>
       <c r="F26" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G26" t="n">
-        <v>22.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>12.0</v>
+        <v>11.5</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C27" t="n">
-        <v>11.0</v>
+        <v>25.0</v>
       </c>
       <c r="D27"/>
       <c r="E27" t="n">
         <v>12.0</v>
       </c>
       <c r="F27" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G27" t="n">
-        <v>20.0</v>
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>